<commit_message>
Format order of events into balanced 2-page document with bilingual notes and Secretary signature
</commit_message>
<xml_diff>
--- a/mysuru_district_athletics_meet_2026_schedule.xlsx
+++ b/mysuru_district_athletics_meet_2026_schedule.xlsx
@@ -5,14 +5,13 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Event Schedule" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Read Me" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="107">
   <si>
     <t>KARNATAKA ATHLETICS ASSOCIATION</t>
   </si>
@@ -29,7 +28,7 @@
     <t>📍 VENUE: Chamundi Vihar Stadium, Mysuru   |   📅 DATE: 31 October 2026   |   ⏰ REPORTING: 8:30 AM</t>
   </si>
   <si>
-    <t>OFFICIAL EVENT SCHEDULE &amp; TIMELINE</t>
+    <t>OFFICIAL ORDER OF EVENTS — MORNING SESSION</t>
   </si>
   <si>
     <t>S. No.</t>
@@ -197,6 +196,9 @@
     <t>12:35 PM</t>
   </si>
   <si>
+    <t>OFFICIAL ORDER OF EVENTS — AFTERNOON SESSION</t>
+  </si>
+  <si>
     <t>12:40 PM</t>
   </si>
   <si>
@@ -299,63 +301,46 @@
     <t>Pentathlon 5/F</t>
   </si>
   <si>
-    <t>IMPORTANT INSTRUCTIONS FOR PARTICIPANTS &amp; TEAM MANAGERS</t>
-  </si>
-  <si>
-    <t>1. Bib Distribution: Strictly on 30 October 2026 from 4:00 PM to 6:00 PM at Chamundi Vihar Stadium. No bibs distributed on 31st Oct.</t>
-  </si>
-  <si>
-    <t>2. Reporting: All athletes must report to the Marshalling Area 30 minutes before the scheduled time of their respective event.</t>
-  </si>
-  <si>
-    <t>3. AFI Rules &amp; Age Verification: Age verification is mandatory. Any over-age athlete will be disqualified immediately.</t>
-  </si>
-  <si>
-    <t>4. NIDJAM Selection: Top performers possessing valid AFI UID will be selected to represent Mysore District at 20th NIDJAM 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hon. Secretary
+    <t>NOTE:</t>
+  </si>
+  <si>
+    <t>ಪ್ರಮುಖ ಸೂಚನೆಗಳು:</t>
+  </si>
+  <si>
+    <t>• Order of events subject to alteration</t>
+  </si>
+  <si>
+    <t>• ಸ್ಪರ್ಧೆಗಳ ಕ್ರಮದಲ್ಲಿ ಬದಲಾವಣೆ ಆಗಬಹುದು</t>
+  </si>
+  <si>
+    <t>• Time may be preponed / postponed - Listen to announcement</t>
+  </si>
+  <si>
+    <t>• ಸ್ಪರ್ಧೆಯ ಸಮಯ ಮುಂದೂಡಬಹುದು ಅಥವಾ ಮೊದಲೇ ನಡೆಸಬಹುದು</t>
+  </si>
+  <si>
+    <t>• Athletes should not leave the stadium during competition</t>
+  </si>
+  <si>
+    <t>• ಎಲ್ಲಾ ಮಾಹಿತಿಯನ್ನು ಅನೌನ್ಸರ್ ಮೂಲಕ ನೀಡಲಾಗುವುದು</t>
+  </si>
+  <si>
+    <t>• Mandatory reporting: 30 minutes prior to scheduled event</t>
+  </si>
+  <si>
+    <t>• ಕ್ರೀಡಾಪಟುಗಳು ಸ್ಪರ್ಧೆಯ ಸಮಯದಲ್ಲಿ ಎಲ್ಲಿಗೂ ಹೋಗಬಾರದು</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Srikanth
+Secretary
 Mysore District Athletics Association</t>
-  </si>
-  <si>
-    <t>Transcription &amp; Meet Notes</t>
-  </si>
-  <si>
-    <t>Purpose</t>
-  </si>
-  <si>
-    <t>Official transcribed schedule for Mysore District Athletics Meet 2026.</t>
-  </si>
-  <si>
-    <t>Affiliation</t>
-  </si>
-  <si>
-    <t>Karnataka Athletics Association (KAA) &amp; Mysore District Athletics Association (MDAA)</t>
-  </si>
-  <si>
-    <t>Categories</t>
-  </si>
-  <si>
-    <t>Under-14 (Boys &amp; Girls) and Under-16 (Boys &amp; Girls)</t>
-  </si>
-  <si>
-    <t>Meet Date</t>
-  </si>
-  <si>
-    <t>31 October 2026 | Chamundi Vihar Stadium, Mysuru</t>
-  </si>
-  <si>
-    <t>NIDJAM Selection</t>
-  </si>
-  <si>
-    <t>Athletes selected from this meet will represent Mysore District at 20th NIDJAM 2026 at Woxsen University, Hyderabad (14–16 Nov 2026).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -366,100 +351,60 @@
     <font>
       <b/>
       <color rgb="FF0F273D"/>
-      <sz val="15"/>
+      <sz val="14.5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <color rgb="FF1D4ED8"/>
-      <sz val="13"/>
+      <sz val="12.5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0F172A"/>
-      <sz val="12"/>
+      <sz val="11.5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <i/>
       <color rgb="FF64748B"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E293B"/>
       <sz val="9.5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1E293B"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="12"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="10.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <color rgb="FF475569"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <color rgb="FF0369A1"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF0F172A"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF94A3B8"/>
       <sz val="9.5"/>
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FFBE123C"/>
-      <sz val="9.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF1E293B"/>
-      <sz val="9.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF475569"/>
-      <sz val="9.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color rgb="FF334155"/>
-      <sz val="9.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1D4ED8"/>
-      <sz val="9.5"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFB45309"/>
+      <color rgb="FF0F172A"/>
       <sz val="9.5"/>
       <name val="Arial"/>
     </font>
@@ -470,18 +415,69 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF0F273D"/>
-      <sz val="12"/>
+      <color rgb="FFBE123C"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF1E293B"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF475569"/>
+      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1E3A8A"/>
+      <color rgb="FF1D4ED8"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFB45309"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF991B1B"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF991B1B"/>
+      <sz val="10"/>
+      <name val="Noto Sans Kannada"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E293B"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E293B"/>
+      <sz val="9"/>
+      <name val="Noto Sans Kannada"/>
+    </font>
+    <font>
+      <color rgb="FF1E293B"/>
+      <sz val="9"/>
+      <name val="Noto Sans Kannada"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -515,7 +511,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2E8F0"/>
+        <fgColor rgb="FFFEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -572,7 +573,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -628,7 +629,7 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -640,33 +641,36 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -689,9 +693,9 @@
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>8000</xdr:colOff>
+      <xdr:colOff>7500</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>84000</xdr:rowOff>
+      <xdr:rowOff>78000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1333500" cy="333375"/>
     <xdr:pic>
@@ -728,9 +732,9 @@
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>36000</xdr:colOff>
+      <xdr:colOff>34000</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>28000</xdr:rowOff>
+      <xdr:rowOff>26000</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="685800" cy="685800"/>
     <xdr:pic>
@@ -1092,18 +1096,18 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="1" max="1" width="7.5" customWidth="1"/>
+    <col min="2" max="2" width="13.5" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="7" width="18" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="7" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1112,7 +1116,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1121,7 +1125,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
@@ -1130,7 +1134,7 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" ht="18" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
@@ -1150,8 +1154,8 @@
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
     </row>
-    <row r="6" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -1162,7 +1166,7 @@
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
     </row>
-    <row r="8" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" ht="23" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
@@ -1185,7 +1189,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>1</v>
       </c>
@@ -1208,7 +1212,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="16">
         <v>2</v>
       </c>
@@ -1231,7 +1235,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>3</v>
       </c>
@@ -1254,7 +1258,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="16">
         <v>4</v>
       </c>
@@ -1264,7 +1268,7 @@
       <c r="C12" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="19" t="s">
         <v>15</v>
       </c>
       <c r="E12" s="20" t="s">
@@ -1277,7 +1281,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
         <v>5</v>
       </c>
@@ -1300,7 +1304,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="16">
         <v>6</v>
       </c>
@@ -1310,7 +1314,7 @@
       <c r="C14" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="19" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="20" t="s">
@@ -1323,7 +1327,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>7</v>
       </c>
@@ -1346,7 +1350,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="16">
         <v>8</v>
       </c>
@@ -1359,7 +1363,7 @@
       <c r="D16" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="E16" s="25" t="s">
+      <c r="E16" s="24" t="s">
         <v>23</v>
       </c>
       <c r="F16" s="21" t="s">
@@ -1369,7 +1373,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>9</v>
       </c>
@@ -1392,7 +1396,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="16">
         <v>10</v>
       </c>
@@ -1402,10 +1406,10 @@
       <c r="C18" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="24" t="s">
+      <c r="D18" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="25" t="s">
+      <c r="E18" s="24" t="s">
         <v>37</v>
       </c>
       <c r="F18" s="21" t="s">
@@ -1415,7 +1419,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>11</v>
       </c>
@@ -1438,7 +1442,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="16">
         <v>12</v>
       </c>
@@ -1448,10 +1452,10 @@
       <c r="C20" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="25" t="s">
+      <c r="E20" s="24" t="s">
         <v>37</v>
       </c>
       <c r="F20" s="21" t="s">
@@ -1461,7 +1465,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>13</v>
       </c>
@@ -1471,7 +1475,7 @@
       <c r="C21" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="D21" s="26" t="s">
+      <c r="D21" s="12" t="s">
         <v>43</v>
       </c>
       <c r="E21" s="13" t="s">
@@ -1484,7 +1488,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="16">
         <v>14</v>
       </c>
@@ -1494,7 +1498,7 @@
       <c r="C22" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="19" t="s">
         <v>15</v>
       </c>
       <c r="E22" s="20" t="s">
@@ -1507,7 +1511,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>15</v>
       </c>
@@ -1530,7 +1534,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="24" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="16">
         <v>16</v>
       </c>
@@ -1543,7 +1547,7 @@
       <c r="D24" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E24" s="25" t="s">
+      <c r="E24" s="24" t="s">
         <v>23</v>
       </c>
       <c r="F24" s="21" t="s">
@@ -1553,7 +1557,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>17</v>
       </c>
@@ -1576,7 +1580,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="16">
         <v>18</v>
       </c>
@@ -1586,7 +1590,7 @@
       <c r="C26" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="D26" s="19" t="s">
         <v>15</v>
       </c>
       <c r="E26" s="20" t="s">
@@ -1599,7 +1603,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="27" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>19</v>
       </c>
@@ -1609,7 +1613,7 @@
       <c r="C27" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="12" t="s">
         <v>54</v>
       </c>
       <c r="E27" s="13" t="s">
@@ -1622,7 +1626,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="16">
         <v>20</v>
       </c>
@@ -1632,10 +1636,10 @@
       <c r="C28" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D28" s="24" t="s">
+      <c r="D28" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="25" t="s">
+      <c r="E28" s="24" t="s">
         <v>23</v>
       </c>
       <c r="F28" s="21" t="s">
@@ -1645,7 +1649,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>21</v>
       </c>
@@ -1668,7 +1672,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="16">
         <v>22</v>
       </c>
@@ -1681,7 +1685,7 @@
       <c r="D30" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E30" s="25" t="s">
+      <c r="E30" s="24" t="s">
         <v>37</v>
       </c>
       <c r="F30" s="21" t="s">
@@ -1691,7 +1695,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
         <v>23</v>
       </c>
@@ -1714,7 +1718,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="32" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="16">
         <v>24</v>
       </c>
@@ -1724,10 +1728,10 @@
       <c r="C32" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="24" t="s">
+      <c r="D32" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="25" t="s">
+      <c r="E32" s="24" t="s">
         <v>23</v>
       </c>
       <c r="F32" s="21" t="s">
@@ -1737,265 +1741,253 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="9">
+    <row r="33" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" ht="23" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="9">
         <v>25</v>
       </c>
-      <c r="B33" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="D33" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="E33" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F33" s="14" t="s">
+      <c r="B35" s="10" t="s">
         <v>62</v>
-      </c>
-      <c r="G33" s="15" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="34" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="16">
-        <v>26</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>63</v>
-      </c>
-      <c r="C34" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="D34" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="E34" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="F34" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="G34" s="22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="35" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="9">
-        <v>27</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>66</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D35" s="26" t="s">
+      <c r="D35" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="E35" s="23" t="s">
-        <v>23</v>
+      <c r="E35" s="13" t="s">
+        <v>34</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G35" s="15" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="36" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="16">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="E36" s="25" t="s">
-        <v>23</v>
+        <v>66</v>
+      </c>
+      <c r="E36" s="20" t="s">
+        <v>16</v>
       </c>
       <c r="F36" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="G36" s="27" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="37" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G36" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="9">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D37" s="26" t="s">
+      <c r="D37" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="E37" s="13" t="s">
-        <v>34</v>
+      <c r="E37" s="23" t="s">
+        <v>23</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="G37" s="15" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="38" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="16">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C38" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="D38" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="E38" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G38" s="25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="9">
+        <v>29</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D38" s="19" t="s">
+      <c r="D39" s="12" t="s">
         <v>54</v>
-      </c>
-      <c r="E38" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="F38" s="21" t="s">
-        <v>71</v>
-      </c>
-      <c r="G38" s="27" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="39" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="9">
-        <v>31</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="C39" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D39" s="12" t="s">
-        <v>15</v>
       </c>
       <c r="E39" s="13" t="s">
         <v>34</v>
       </c>
       <c r="F39" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="16">
+        <v>30</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D40" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E40" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F40" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="G40" s="25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="9">
+        <v>31</v>
+      </c>
+      <c r="B41" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="G39" s="15" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="40" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="16">
+      <c r="C41" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E41" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="42" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="16">
         <v>32</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B42" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="C42" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D42" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="E42" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F42" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="C40" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="D40" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="E40" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="F40" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="G40" s="22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="41" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="9">
+      <c r="G42" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="43" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="9">
         <v>33</v>
       </c>
-      <c r="B41" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="C41" s="11" t="s">
+      <c r="B43" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D41" s="26" t="s">
+      <c r="D43" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E43" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F41" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="G41" s="15" t="s">
+      <c r="F43" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G43" s="15" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="42" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="16">
+    <row r="44" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="16">
         <v>34</v>
       </c>
-      <c r="B42" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="C42" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="D42" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="E42" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F42" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="G42" s="22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="43" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="9">
-        <v>35</v>
-      </c>
-      <c r="B43" s="10" t="s">
+      <c r="B44" s="17" t="s">
         <v>81</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D43" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F43" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="G43" s="15" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="44" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="16">
-        <v>36</v>
-      </c>
-      <c r="B44" s="17" t="s">
-        <v>84</v>
       </c>
       <c r="C44" s="18" t="s">
         <v>53</v>
@@ -2003,45 +1995,45 @@
       <c r="D44" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E44" s="20" t="s">
-        <v>16</v>
+      <c r="E44" s="24" t="s">
+        <v>23</v>
       </c>
       <c r="F44" s="21" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="G44" s="22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="45" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C45" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D45" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="E45" s="23" t="s">
-        <v>37</v>
+      <c r="D45" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="E45" s="13" t="s">
+        <v>34</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G45" s="15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="46" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="16">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C46" s="18" t="s">
         <v>53</v>
@@ -2049,8 +2041,8 @@
       <c r="D46" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="E46" s="25" t="s">
-        <v>23</v>
+      <c r="E46" s="20" t="s">
+        <v>16</v>
       </c>
       <c r="F46" s="21" t="s">
         <v>17</v>
@@ -2059,104 +2051,104 @@
         <v>21</v>
       </c>
     </row>
-    <row r="47" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="9">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C47" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D47" s="26" t="s">
+      <c r="D47" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="E47" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="F47" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="G47" s="15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="16">
+        <v>38</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C48" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="D48" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E48" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F48" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="G48" s="22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="9">
+        <v>39</v>
+      </c>
+      <c r="B49" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C49" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E47" s="13" t="s">
+      <c r="E49" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F47" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="G47" s="15" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="48" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="16">
+      <c r="F49" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="G49" s="15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="16">
         <v>40</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B50" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E50" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F50" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="C48" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="D48" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="E48" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F48" s="21" t="s">
-        <v>88</v>
-      </c>
-      <c r="G48" s="22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="49" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="9">
+      <c r="G50" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="9">
         <v>41</v>
       </c>
-      <c r="B49" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D49" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="F49" s="14" t="s">
+      <c r="B51" s="10" t="s">
         <v>91</v>
-      </c>
-      <c r="G49" s="15" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="50" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="16">
-        <v>42</v>
-      </c>
-      <c r="B50" s="17" t="s">
-        <v>92</v>
-      </c>
-      <c r="C50" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D50" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="E50" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="F50" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="G50" s="22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="51" ht="21" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="9">
-        <v>43</v>
-      </c>
-      <c r="B51" s="10" t="s">
-        <v>93</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>14</v>
@@ -2168,151 +2160,156 @@
         <v>34</v>
       </c>
       <c r="F51" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="G51" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="16">
+        <v>42</v>
+      </c>
+      <c r="B52" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E52" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="F52" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="G52" s="22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="53" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="9">
+        <v>43</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="G51" s="15" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="28" t="s">
+      <c r="C53" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="F53" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="B53" s="28"/>
-      <c r="C53" s="28"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="28"/>
-      <c r="F53" s="28"/>
-      <c r="G53" s="28"/>
-    </row>
-    <row r="54" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="29" t="s">
+      <c r="G53" s="15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="55" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="B54" s="29"/>
-      <c r="C54" s="29"/>
-      <c r="D54" s="29"/>
-      <c r="E54" s="29"/>
-      <c r="F54" s="29"/>
-      <c r="G54" s="29"/>
-    </row>
-    <row r="55" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="29" t="s">
+      <c r="B55" s="26"/>
+      <c r="C55" s="26"/>
+      <c r="D55" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="B55" s="29"/>
-      <c r="C55" s="29"/>
-      <c r="D55" s="29"/>
-      <c r="E55" s="29"/>
-      <c r="F55" s="29"/>
-      <c r="G55" s="29"/>
-    </row>
-    <row r="56" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="29" t="s">
+      <c r="E55" s="27"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="27"/>
+    </row>
+    <row r="56" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="28" t="s">
         <v>98</v>
       </c>
-      <c r="B56" s="29"/>
-      <c r="C56" s="29"/>
-      <c r="D56" s="29"/>
+      <c r="B56" s="28"/>
+      <c r="C56" s="28"/>
+      <c r="D56" s="29" t="s">
+        <v>99</v>
+      </c>
       <c r="E56" s="29"/>
       <c r="F56" s="29"/>
       <c r="G56" s="29"/>
     </row>
-    <row r="57" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="B57" s="29"/>
-      <c r="C57" s="29"/>
-      <c r="D57" s="29"/>
-      <c r="E57" s="29"/>
-      <c r="F57" s="29"/>
-      <c r="G57" s="29"/>
-    </row>
-    <row r="59" ht="36" customHeight="1" spans="5:7" x14ac:dyDescent="0.25">
-      <c r="E59" s="30" t="s">
+    <row r="57" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="F59" s="30"/>
-      <c r="G59" s="30"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="30"/>
+      <c r="D57" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="E57" s="31"/>
+      <c r="F57" s="31"/>
+      <c r="G57" s="31"/>
+    </row>
+    <row r="58" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="B58" s="30"/>
+      <c r="C58" s="30"/>
+      <c r="D58" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="E58" s="31"/>
+      <c r="F58" s="31"/>
+      <c r="G58" s="31"/>
+    </row>
+    <row r="59" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="B59" s="30"/>
+      <c r="C59" s="30"/>
+      <c r="D59" s="31" t="s">
+        <v>105</v>
+      </c>
+      <c r="E59" s="31"/>
+      <c r="F59" s="31"/>
+      <c r="G59" s="31"/>
+    </row>
+    <row r="61" ht="42" customHeight="1" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E61" s="32" t="s">
+        <v>106</v>
+      </c>
+      <c r="F61" s="32"/>
+      <c r="G61" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="18">
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A53:G53"/>
-    <mergeCell ref="A54:G54"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A56:G56"/>
-    <mergeCell ref="A57:G57"/>
-    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A55:C55"/>
+    <mergeCell ref="D55:G55"/>
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="D56:G56"/>
+    <mergeCell ref="A57:C57"/>
+    <mergeCell ref="D57:G57"/>
+    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="D58:G58"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="D59:G59"/>
+    <mergeCell ref="E61:G61"/>
   </mergeCells>
-  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageMargins left="0.35" right="0.35" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="33" max="16838" man="1"/>
+  </rowBreaks>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="70" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="32" t="s">
-        <v>106</v>
-      </c>
-      <c r="B5" s="33" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="B6" s="33" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="32" t="s">
-        <v>110</v>
-      </c>
-      <c r="B7" s="33" t="s">
-        <v>111</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>